<commit_message>
Added multi-license testcase grouping for deeplink tests
</commit_message>
<xml_diff>
--- a/testcases/deeplinks/deeplink_tests.xlsx
+++ b/testcases/deeplinks/deeplink_tests.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marnisaisanjay/Documents/personalprojects/AppPilot/testcases/deeplinks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF27124A-0E22-204B-B7F0-B597C8E06334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39639B2-8181-7446-AF52-2E263D49BEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{C5943666-9D12-0C47-8784-2B49B0DE6ECC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="67">
   <si>
     <t>Premium</t>
   </si>
@@ -72,13 +72,181 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>Enterprise</t>
+  </si>
+  <si>
+    <t>TC005</t>
+  </si>
+  <si>
+    <t>Trial</t>
+  </si>
+  <si>
+    <t>TC006</t>
+  </si>
+  <si>
+    <t>Developer</t>
+  </si>
+  <si>
+    <t>TC007</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
+    <t>TC010</t>
+  </si>
+  <si>
+    <t>TC011</t>
+  </si>
+  <si>
+    <t>TC012</t>
+  </si>
+  <si>
+    <t>TC013</t>
+  </si>
+  <si>
+    <t>TC014</t>
+  </si>
+  <si>
+    <t>TC015</t>
+  </si>
+  <si>
+    <t>TC016</t>
+  </si>
+  <si>
+    <t>TC017</t>
+  </si>
+  <si>
+    <t>TC018</t>
+  </si>
+  <si>
+    <t>TC019</t>
+  </si>
+  <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>TC026</t>
+  </si>
+  <si>
+    <t>TC027</t>
+  </si>
+  <si>
+    <t>TC028</t>
+  </si>
+  <si>
+    <t>TC029</t>
+  </si>
+  <si>
+    <t>TC030</t>
+  </si>
+  <si>
+    <t>TC031</t>
+  </si>
+  <si>
+    <t>TC032</t>
+  </si>
+  <si>
+    <t>TC033</t>
+  </si>
+  <si>
+    <t>TC034</t>
+  </si>
+  <si>
+    <t>TC035</t>
+  </si>
+  <si>
+    <t>TC036</t>
+  </si>
+  <si>
+    <t>TC037</t>
+  </si>
+  <si>
+    <t>TC038</t>
+  </si>
+  <si>
+    <t>TC039</t>
+  </si>
+  <si>
+    <t>TC040</t>
+  </si>
+  <si>
+    <t>TC041</t>
+  </si>
+  <si>
+    <t>TC042</t>
+  </si>
+  <si>
+    <t>TC043</t>
+  </si>
+  <si>
+    <t>TC044</t>
+  </si>
+  <si>
+    <t>TC045</t>
+  </si>
+  <si>
+    <t>TC046</t>
+  </si>
+  <si>
+    <t>TC047</t>
+  </si>
+  <si>
+    <t>TC048</t>
+  </si>
+  <si>
+    <t>TC049</t>
+  </si>
+  <si>
+    <t>TC050</t>
+  </si>
+  <si>
+    <t>TC051</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -90,6 +258,14 @@
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -132,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -144,6 +320,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -164,6 +343,9 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -185,15 +367,19 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C3E0EAF0-8322-9943-9361-9A2C145B69AC}" name="TestCasesTable" displayName="TestCasesTable" ref="A2:E4" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A2:E4" xr:uid="{C3E0EAF0-8322-9943-9361-9A2C145B69AC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C3E0EAF0-8322-9943-9361-9A2C145B69AC}" name="TestCasesTable" displayName="TestCasesTable" ref="A2:E53" totalsRowShown="0" headerRowDxfId="4" dataDxfId="6">
+  <autoFilter ref="A2:E53" xr:uid="{C3E0EAF0-8322-9943-9361-9A2C145B69AC}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{E7C93395-3D2D-F24C-B14C-2E0B10E9B5B2}" name="Test Case ID" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{1C1E9B71-D984-1A45-98E8-18E5C9778295}" name="Launch URL" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{E7C93395-3D2D-F24C-B14C-2E0B10E9B5B2}" name="Test Case ID" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{1C1E9B71-D984-1A45-98E8-18E5C9778295}" name="Launch URL" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{6CC5405F-8922-2E4C-B7D1-5D204DC658A0}" name="License" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{F4FB8A81-E7AB-BA43-8829-4FE851CDEED2}" name="Expected Screen" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{0D6DC78D-E6A7-C946-892F-2EF1D0741508}" name="Installed" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{F4FB8A81-E7AB-BA43-8829-4FE851CDEED2}" name="Expected Screen" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{0D6DC78D-E6A7-C946-892F-2EF1D0741508}" name="Installed" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -516,17 +702,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B78DF14-4F71-D549-86BA-243B67A56556}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="34.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="34.6640625" style="1"/>
-    <col min="2" max="2" width="138.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" style="1"/>
-    <col min="4" max="4" width="40.33203125" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="34.6640625" style="1"/>
+    <col min="1" max="1" width="15" style="1" customWidth="1"/>
+    <col min="2" max="2" width="46.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="60" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="34.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="24" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
@@ -535,24 +722,24 @@
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" s="2" customFormat="1" ht="272" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -569,10 +756,858 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:5" s="2" customFormat="1" ht="123" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="6" spans="1:5" s="2" customFormat="1" ht="71" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D6" s="3"/>
+    <row r="4" spans="1:5" s="2" customFormat="1" ht="272" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" ht="272" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" ht="272" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="272" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D54" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>